<commit_message>
feat(fy27q3): sort stock table by entry date, pick up 2 new result announcements
Quarter position-taking table now sorts by entry date ascending (unannounced
stocks pushed to the end) instead of raw JSON order.

Live NSE fetch picked up 2 results announced since yesterday's scrape:
JIOFIN (15-Oct-2026) and KOTAKBANK (24-Oct-2026, a Saturday filing). Updated
their dates and the quarter's announced/pending counts (24/27 -> 26/25).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nifty50_Upcoming_Quarterly_Result_Dates_2026.xlsx
+++ b/Nifty50_Upcoming_Quarterly_Result_Dates_2026.xlsx
@@ -1642,22 +1642,22 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Expected: 18-Oct</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Pending Announcement (Est: Oct-Nov)</t>
+          <t>ANNOUNCED ON NSE ✅</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Q2 FY27 Financial Results (Period ended Sept 30)</t>
+          <t>Financial Results</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Historically announced around 18-Oct</t>
+          <t>To consider and approve the unaudited financial results for the quarter and half year ended September 30, 2026</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1732,22 +1732,22 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Expected: 19-Oct</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Pending Announcement (Est: Oct-Nov)</t>
+          <t>ANNOUNCED ON NSE ✅</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Q2 FY27 Financial Results (Period ended Sept 30)</t>
+          <t>Financial Results</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Historically announced around 19-Oct</t>
+          <t>To consider and approve the Standalone and Consolidated Unaudited Financial Results for the quarter and half year ended September 30, 2026</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">

</xml_diff>